<commit_message>
Renombrar archivos segun METADATOS y regenerar matriz
</commit_message>
<xml_diff>
--- a/trazabilidad/Matriz_de_trazabilidad.xlsx
+++ b/trazabilidad/Matriz_de_trazabilidad.xlsx
@@ -2332,7 +2332,7 @@
     <row r="34" ht="31" customHeight="1" s="36">
       <c r="A34" s="115" t="inlineStr">
         <is>
-          <t>Generada el 2026-09-21 con trazabilidad/generar_matriz.py sobre el commit e915f54 (con cambios sin confirmar). 13 pruebas automáticas ejecutadas. No edites las hojas a mano: cambia el repositorio y vuelve a ejecutar el script.</t>
+          <t>Generada el 2026-09-21 con trazabilidad/generar_matriz.py sobre el commit c43e63b (con cambios sin confirmar). 13 pruebas automáticas ejecutadas. No edites las hojas a mano: cambia el repositorio y vuelve a ejecutar el script.</t>
         </is>
       </c>
       <c r="B34" s="115" t="n"/>
@@ -4515,7 +4515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="36" min="1" max="1"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1" s="36">
+    <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="38" t="n">
         <v>1</v>
       </c>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="C3" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Metadatos incompletos</t>
         </is>
       </c>
       <c r="D3" s="38" t="inlineStr">
@@ -4586,16 +4586,16 @@
       </c>
       <c r="E3" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/Product_Backlog_Priorizado.docx no está en el repositorio.</t>
+          <t>Falta o está pendiente: fecha de cierre.</t>
         </is>
       </c>
       <c r="F3" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1" s="36">
+          <t>Completar el encabezado del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="36">
       <c r="A4" s="38" t="n">
         <v>2</v>
       </c>
@@ -4606,26 +4606,26 @@
       </c>
       <c r="C4" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Metadatos incompletos</t>
         </is>
       </c>
       <c r="D4" s="38" t="inlineStr">
         <is>
-          <t>C1-RFC-A1</t>
+          <t>C1-VB</t>
         </is>
       </c>
       <c r="E4" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/RFC-A1_Clima_Extremo.docx no está en el repositorio.</t>
+          <t>Falta o está pendiente: fecha de cierre.</t>
         </is>
       </c>
       <c r="F4" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1" s="36">
+          <t>Completar el encabezado del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="36">
       <c r="A5" s="38" t="n">
         <v>3</v>
       </c>
@@ -4636,26 +4636,26 @@
       </c>
       <c r="C5" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Metadatos incompletos</t>
         </is>
       </c>
       <c r="D5" s="38" t="inlineStr">
         <is>
-          <t>C1-RFC-A2</t>
+          <t>DOC-VAL</t>
         </is>
       </c>
       <c r="E5" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/RFC-A2_Notificaciones.docx no está en el repositorio.</t>
+          <t>Falta o está pendiente: fecha de cierre.</t>
         </is>
       </c>
       <c r="F5" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1" s="36">
+          <t>Completar el encabezado del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="36">
       <c r="A6" s="38" t="n">
         <v>4</v>
       </c>
@@ -4666,22 +4666,22 @@
       </c>
       <c r="C6" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Metadatos incompletos</t>
         </is>
       </c>
       <c r="D6" s="38" t="inlineStr">
         <is>
-          <t>C1-RFC-B1</t>
+          <t>TEST-MANUAL</t>
         </is>
       </c>
       <c r="E6" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/RFC-B1_Criterio_Puntuacion.docx no está en el repositorio.</t>
+          <t>Falta o está pendiente: fecha de cierre.</t>
         </is>
       </c>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
+          <t>Completar el encabezado del archivo.</t>
         </is>
       </c>
     </row>
@@ -4689,29 +4689,29 @@
       <c r="A7" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
       <c r="C7" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Cambio propuesto sin RFC</t>
         </is>
       </c>
       <c r="D7" s="38" t="inlineStr">
         <is>
-          <t>C1-RFC-B2</t>
+          <t>CA1–CA5</t>
         </is>
       </c>
       <c r="E7" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/RFC-B2_Formula_Hibrida.docx no está en el repositorio.</t>
+          <t>La sección 6 propone reformular los criterios de aceptación, pero no hay una RFC que registre el cambio.</t>
         </is>
       </c>
       <c r="F7" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
+          <t>Registrar la RFC (formulario del curso) y agregarla al registro.</t>
         </is>
       </c>
     </row>
@@ -4719,29 +4719,29 @@
       <c r="A8" s="38" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
       <c r="C8" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Criterio de aceptación sin requisito</t>
         </is>
       </c>
       <c r="D8" s="38" t="inlineStr">
         <is>
-          <t>C1-RFC-C1</t>
+          <t>CA5</t>
         </is>
       </c>
       <c r="E8" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/RFC-C1_IA_Predictiva.docx no está en el repositorio.</t>
+          <t>Está propuesto en la sección 6 del documento, pero ningún requisito de la sección 2 lo usa; por eso no tiene código ni pruebas.</t>
         </is>
       </c>
       <c r="F8" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
+          <t>Crear el requisito que lo cubra.</t>
         </is>
       </c>
     </row>
@@ -4749,29 +4749,29 @@
       <c r="A9" s="38" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
       <c r="C9" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Escenarios manuales sin ejecutar</t>
         </is>
       </c>
       <c r="D9" s="38" t="inlineStr">
         <is>
-          <t>C1-VB</t>
+          <t>TEST-MANUAL</t>
         </is>
       </c>
       <c r="E9" s="38" t="inlineStr">
         <is>
-          <t>caso1-aerea/Product_Vision_Board.docx no está en el repositorio.</t>
+          <t>Pendientes: TC-M1, TC-M2, TC-M3, TC-M4, TC-M5.</t>
         </is>
       </c>
       <c r="F9" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
+          <t>Ejecutarlos y anotar resultado, fecha y observaciones.</t>
         </is>
       </c>
     </row>
@@ -4779,29 +4779,29 @@
       <c r="A10" s="38" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
       <c r="C10" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Requisito sin prueba ejecutada</t>
         </is>
       </c>
       <c r="D10" s="38" t="inlineStr">
         <is>
-          <t>C2-SRS</t>
+          <t>RF-A5</t>
         </is>
       </c>
       <c r="E10" s="38" t="inlineStr">
         <is>
-          <t>caso2-simulador/SRS_Simulador_Transmision_Mecanica.docx no está en el repositorio.</t>
+          <t>Sus pruebas (TC-M4, TC-M5) siguen en «Pendiente».</t>
         </is>
       </c>
       <c r="F10" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
+          <t>Ejecutarlas y registrar el resultado en tests/escenarios_manuales.md.</t>
         </is>
       </c>
     </row>
@@ -4809,387 +4809,117 @@
       <c r="A11" s="38" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Media</t>
         </is>
       </c>
       <c r="C11" s="38" t="inlineStr">
         <is>
-          <t>Archivo declarado no existe</t>
+          <t>Requisito sin prueba ejecutada</t>
         </is>
       </c>
       <c r="D11" s="38" t="inlineStr">
         <is>
-          <t>C2-TC</t>
+          <t>RNF-1</t>
         </is>
       </c>
       <c r="E11" s="38" t="inlineStr">
         <is>
-          <t>caso2-simulador/Test_Case_Simulador_Transmision.docx no está en el repositorio.</t>
+          <t>Sus pruebas (TC-M4) siguen en «Pendiente».</t>
         </is>
       </c>
       <c r="F11" s="38" t="inlineStr">
         <is>
-          <t>Copiar el archivo a esa carpeta con ese nombre, o corregir la columna «Archivo» de METADATOS.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1" s="36">
+          <t>Ejecutarlas y registrar el resultado en tests/escenarios_manuales.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="31" customHeight="1" s="36">
       <c r="A12" s="38" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Baja</t>
         </is>
       </c>
       <c r="C12" s="38" t="inlineStr">
         <is>
-          <t>Metadatos incompletos</t>
+          <t>Código sin requisito</t>
         </is>
       </c>
       <c r="D12" s="38" t="inlineStr">
         <is>
-          <t>C1-BACKLOG</t>
+          <t>caso3-dietas/src/screens/Login.jsx</t>
         </is>
       </c>
       <c r="E12" s="38" t="inlineStr">
         <is>
-          <t>Falta o está pendiente: fecha de cierre.</t>
+          <t>Implementa comportamiento que ningún requisito de la sección 2 respalda.</t>
         </is>
       </c>
       <c r="F12" s="38" t="inlineStr">
         <is>
-          <t>Completar el encabezado del archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1" s="36">
+          <t>Asociarlo a un requisito, o marcarlo con la etiqueta de infraestructura si no aplica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="31" customHeight="1" s="36">
       <c r="A13" s="38" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Baja</t>
         </is>
       </c>
       <c r="C13" s="38" t="inlineStr">
         <is>
-          <t>Metadatos incompletos</t>
+          <t>ID de requisito no definido en el documento</t>
         </is>
       </c>
       <c r="D13" s="38" t="inlineStr">
         <is>
-          <t>C1-VB</t>
+          <t>RF1–RF5</t>
         </is>
       </c>
       <c r="E13" s="38" t="inlineStr">
         <is>
-          <t>Falta o está pendiente: fecha de cierre.</t>
+          <t>Citado en caso3-dietas/src/screens/Catalog.jsx, pero la sección 2 de caso3-dietas/docs/Documento_de_validacion.md no lo define.</t>
         </is>
       </c>
       <c r="F13" s="38" t="inlineStr">
         <is>
-          <t>Completar el encabezado del archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" s="36">
+          <t>Definir el requisito en el documento (o quitar la etiqueta si está fuera de alcance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="31" customHeight="1" s="36">
       <c r="A14" s="38" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Baja</t>
         </is>
       </c>
       <c r="C14" s="38" t="inlineStr">
         <is>
-          <t>Metadatos incompletos</t>
+          <t>Requisito ausente en la aplicación</t>
         </is>
       </c>
       <c r="D14" s="38" t="inlineStr">
         <is>
-          <t>DOC-VAL</t>
+          <t>RNF-1</t>
         </is>
       </c>
       <c r="E14" s="38" t="inlineStr">
         <is>
-          <t>Falta o está pendiente: fecha de cierre.</t>
+          <t>Está en el documento pero no en la pantalla «Objetivo» (caso3-dietas/src/screens/About.jsx).</t>
         </is>
       </c>
       <c r="F14" s="38" t="inlineStr">
-        <is>
-          <t>Completar el encabezado del archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1" s="36">
-      <c r="A15" s="38" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="C15" s="38" t="inlineStr">
-        <is>
-          <t>Metadatos incompletos</t>
-        </is>
-      </c>
-      <c r="D15" s="38" t="inlineStr">
-        <is>
-          <t>TEST-MANUAL</t>
-        </is>
-      </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>Falta o está pendiente: fecha de cierre.</t>
-        </is>
-      </c>
-      <c r="F15" s="38" t="inlineStr">
-        <is>
-          <t>Completar el encabezado del archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="31" customHeight="1" s="36">
-      <c r="A16" s="38" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="38" t="inlineStr">
-        <is>
-          <t>Cambio propuesto sin RFC</t>
-        </is>
-      </c>
-      <c r="D16" s="38" t="inlineStr">
-        <is>
-          <t>CA1–CA5</t>
-        </is>
-      </c>
-      <c r="E16" s="38" t="inlineStr">
-        <is>
-          <t>La sección 6 propone reformular los criterios de aceptación, pero no hay una RFC que registre el cambio.</t>
-        </is>
-      </c>
-      <c r="F16" s="38" t="inlineStr">
-        <is>
-          <t>Registrar la RFC (formulario del curso) y agregarla al registro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="31" customHeight="1" s="36">
-      <c r="A17" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C17" s="38" t="inlineStr">
-        <is>
-          <t>Criterio de aceptación sin requisito</t>
-        </is>
-      </c>
-      <c r="D17" s="38" t="inlineStr">
-        <is>
-          <t>CA5</t>
-        </is>
-      </c>
-      <c r="E17" s="38" t="inlineStr">
-        <is>
-          <t>Está propuesto en la sección 6 del documento, pero ningún requisito de la sección 2 lo usa; por eso no tiene código ni pruebas.</t>
-        </is>
-      </c>
-      <c r="F17" s="38" t="inlineStr">
-        <is>
-          <t>Crear el requisito que lo cubra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="31" customHeight="1" s="36">
-      <c r="A18" s="38" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C18" s="38" t="inlineStr">
-        <is>
-          <t>Escenarios manuales sin ejecutar</t>
-        </is>
-      </c>
-      <c r="D18" s="38" t="inlineStr">
-        <is>
-          <t>TEST-MANUAL</t>
-        </is>
-      </c>
-      <c r="E18" s="38" t="inlineStr">
-        <is>
-          <t>Pendientes: TC-M1, TC-M2, TC-M3, TC-M4, TC-M5.</t>
-        </is>
-      </c>
-      <c r="F18" s="38" t="inlineStr">
-        <is>
-          <t>Ejecutarlos y anotar resultado, fecha y observaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="31" customHeight="1" s="36">
-      <c r="A19" s="38" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C19" s="38" t="inlineStr">
-        <is>
-          <t>Requisito sin prueba ejecutada</t>
-        </is>
-      </c>
-      <c r="D19" s="38" t="inlineStr">
-        <is>
-          <t>RF-A5</t>
-        </is>
-      </c>
-      <c r="E19" s="38" t="inlineStr">
-        <is>
-          <t>Sus pruebas (TC-M4, TC-M5) siguen en «Pendiente».</t>
-        </is>
-      </c>
-      <c r="F19" s="38" t="inlineStr">
-        <is>
-          <t>Ejecutarlas y registrar el resultado en tests/escenarios_manuales.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="31" customHeight="1" s="36">
-      <c r="A20" s="38" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C20" s="38" t="inlineStr">
-        <is>
-          <t>Requisito sin prueba ejecutada</t>
-        </is>
-      </c>
-      <c r="D20" s="38" t="inlineStr">
-        <is>
-          <t>RNF-1</t>
-        </is>
-      </c>
-      <c r="E20" s="38" t="inlineStr">
-        <is>
-          <t>Sus pruebas (TC-M4) siguen en «Pendiente».</t>
-        </is>
-      </c>
-      <c r="F20" s="38" t="inlineStr">
-        <is>
-          <t>Ejecutarlas y registrar el resultado en tests/escenarios_manuales.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="31" customHeight="1" s="36">
-      <c r="A21" s="38" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C21" s="38" t="inlineStr">
-        <is>
-          <t>Código sin requisito</t>
-        </is>
-      </c>
-      <c r="D21" s="38" t="inlineStr">
-        <is>
-          <t>caso3-dietas/src/screens/Login.jsx</t>
-        </is>
-      </c>
-      <c r="E21" s="38" t="inlineStr">
-        <is>
-          <t>Implementa comportamiento que ningún requisito de la sección 2 respalda.</t>
-        </is>
-      </c>
-      <c r="F21" s="38" t="inlineStr">
-        <is>
-          <t>Asociarlo a un requisito, o marcarlo con la etiqueta de infraestructura si no aplica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="31" customHeight="1" s="36">
-      <c r="A22" s="38" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C22" s="38" t="inlineStr">
-        <is>
-          <t>ID de requisito no definido en el documento</t>
-        </is>
-      </c>
-      <c r="D22" s="38" t="inlineStr">
-        <is>
-          <t>RF1–RF5</t>
-        </is>
-      </c>
-      <c r="E22" s="38" t="inlineStr">
-        <is>
-          <t>Citado en caso3-dietas/src/screens/Catalog.jsx, pero la sección 2 de caso3-dietas/docs/Documento_de_validacion.md no lo define.</t>
-        </is>
-      </c>
-      <c r="F22" s="38" t="inlineStr">
-        <is>
-          <t>Definir el requisito en el documento (o quitar la etiqueta si está fuera de alcance).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="31" customHeight="1" s="36">
-      <c r="A23" s="38" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C23" s="38" t="inlineStr">
-        <is>
-          <t>Requisito ausente en la aplicación</t>
-        </is>
-      </c>
-      <c r="D23" s="38" t="inlineStr">
-        <is>
-          <t>RNF-1</t>
-        </is>
-      </c>
-      <c r="E23" s="38" t="inlineStr">
-        <is>
-          <t>Está en el documento pero no en la pantalla «Objetivo» (caso3-dietas/src/screens/About.jsx).</t>
-        </is>
-      </c>
-      <c r="F23" s="38" t="inlineStr">
         <is>
           <t>Agregarlo a la lista de requisitos de la pantalla.</t>
         </is>
@@ -5501,7 +5231,7 @@
       </c>
       <c r="F3" s="13" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5615,7 +5345,7 @@
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5672,7 +5402,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5729,7 +5459,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5786,7 +5516,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5843,7 +5573,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5957,7 +5687,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -6014,7 +5744,7 @@
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -6071,7 +5801,7 @@
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">

</xml_diff>